<commit_message>
Nova atualização do benefício
</commit_message>
<xml_diff>
--- a/TesteOdair.xlsx
+++ b/TesteOdair.xlsx
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B2" s="1">
         <f>Planilha3!B1</f>
-        <v>7605</v>
+        <v>7718</v>
       </c>
       <c r="C2" s="2">
         <v>45867</v>
@@ -1160,7 +1160,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="12.6761904761905" defaultRowHeight="12.8" customHeight="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" ht="12.75" spans="1:2">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B1">
         <f>SUM(A2:A36)</f>
-        <v>7605</v>
+        <v>7718</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:1">
@@ -1230,6 +1230,11 @@
     <row r="13" customHeight="1" spans="1:1">
       <c r="A13">
         <v>108</v>
+      </c>
+    </row>
+    <row r="14" customHeight="1" spans="1:1">
+      <c r="A14">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nova atualização no benefício
</commit_message>
<xml_diff>
--- a/TesteOdair.xlsx
+++ b/TesteOdair.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B2" s="4">
         <f>Planilha3!B1</f>
-        <v>9497</v>
+        <v>9608</v>
       </c>
       <c r="C2" s="5">
         <v>45867</v>
@@ -1169,7 +1169,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultColWidth="12.6761904761905" defaultRowHeight="12.8" customHeight="1" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.6761904761905" style="1"/>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B1" s="2">
         <f>SUM(A2:A54)</f>
-        <v>9497</v>
+        <v>9608</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:1">
@@ -1322,6 +1322,11 @@
     <row r="29" customHeight="1" spans="1:1">
       <c r="A29" s="1">
         <v>134</v>
+      </c>
+    </row>
+    <row r="30" customHeight="1" spans="1:1">
+      <c r="A30" s="1">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nova atualização do beneficiamento
</commit_message>
<xml_diff>
--- a/TesteOdair.xlsx
+++ b/TesteOdair.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B2" s="4">
         <f>Planilha3!B1</f>
-        <v>9867</v>
+        <v>9996</v>
       </c>
       <c r="C2" s="5">
         <v>45867</v>
@@ -1169,7 +1169,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultColWidth="12.6761904761905" defaultRowHeight="12.8" customHeight="1" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.6761904761905" style="1"/>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B1" s="2">
         <f>SUM(A2:A54)</f>
-        <v>9867</v>
+        <v>9996</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:1">
@@ -1336,6 +1336,11 @@
     </row>
     <row r="32" customHeight="1" spans="1:1">
       <c r="A32" s="1">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customHeight="1" spans="1:1">
+      <c r="A33" s="1">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalizada - Fim da Safra 24/25
</commit_message>
<xml_diff>
--- a/TesteOdair.xlsx
+++ b/TesteOdair.xlsx
@@ -1146,11 +1146,11 @@
     </row>
     <row r="2" customHeight="1" spans="1:3">
       <c r="A2" s="4">
-        <v>11278</v>
+        <v>11286</v>
       </c>
       <c r="B2" s="4">
         <f>Planilha3!B1</f>
-        <v>11186</v>
+        <v>11286</v>
       </c>
       <c r="C2" s="5">
         <v>45867</v>
@@ -1169,7 +1169,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr defaultColWidth="12.6761904761905" defaultRowHeight="12.8" customHeight="1" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.6761904761905" style="1"/>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B1" s="2">
         <f>SUM(A2:A54)</f>
-        <v>11186</v>
+        <v>11286</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:1">
@@ -1387,6 +1387,11 @@
     <row r="42" customHeight="1" spans="1:1">
       <c r="A42" s="1">
         <v>98</v>
+      </c>
+    </row>
+    <row r="43" customHeight="1" spans="1:1">
+      <c r="A43" s="1">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>